<commit_message>
docs(tests): rewrite TC-010 to match actual behaviour
The case assumed the registration form offered a Veterinarian option, so it was
not executable as written. RegisterPage restricts the schema to
pet-owner|admin, and the API independently returns 403 for a direct attempt.

TC-010 now verifies both layers: that the UI omits the option, and that the API
rejects a request crafted to bypass it. Verified live - 403 'Veterinarian
accounts are created by an administrator', no account created.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TEST_CASES.xlsx
+++ b/docs/TEST_CASES.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -14,14 +13,14 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Cases'!$A$1:$J$124</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,16 +29,28 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF00B050"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="11">
@@ -51,47 +62,47 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="FF1F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EAF3FA"/>
+        <fgColor rgb="FFEAF3FA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDF7ED"/>
+        <fgColor rgb="FFEDF7ED"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF8E7"/>
+        <fgColor rgb="FFFFF8E7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDEEF0"/>
+        <fgColor rgb="FFFDEEF0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F3EEF9"/>
+        <fgColor rgb="FFF3EEF9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EAF7F7"/>
+        <fgColor rgb="FFEAF7F7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3E8"/>
+        <fgColor rgb="FFFFF3E8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0F0F5"/>
+        <fgColor rgb="FFF0F0F5"/>
       </patternFill>
     </fill>
   </fills>
@@ -105,23 +116,24 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -185,9 +197,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -551,13 +566,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="18" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Test Execution Summary</t>
@@ -606,7 +621,6 @@
           <t>Tested by</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -614,7 +628,6 @@
           <t>Date</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -622,7 +635,6 @@
           <t>Build / commit</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -726,7 +738,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J124"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -792,7 +804,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="43.2" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
           <t>TC-001</t>
@@ -830,15 +842,15 @@
           <t>All 13 containers reach Up state</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr"/>
+      <c r="H2" s="6" t="n"/>
       <c r="I2" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J2" s="6" t="inlineStr"/>
-    </row>
-    <row r="3">
+      <c r="J2" s="6" t="n"/>
+    </row>
+    <row r="3" ht="28.8" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>TC-002</t>
@@ -875,13 +887,13 @@
           <t>Each returns {"status":"ok"}</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr"/>
+      <c r="H3" s="6" t="n"/>
       <c r="I3" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J3" s="6" t="inlineStr"/>
+      <c r="J3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -919,15 +931,15 @@
           <t>Landing page renders without console errors</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr"/>
+      <c r="H4" s="6" t="n"/>
       <c r="I4" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr"/>
-    </row>
-    <row r="5">
+      <c r="J4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="28.8" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>TC-004</t>
@@ -963,15 +975,15 @@
           <t>available=true; 20 diseases, 24 symptoms, 8 vaccines, 48 INDICATES, 12 PREVENTS</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="n"/>
       <c r="I5" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr"/>
-    </row>
-    <row r="6">
+      <c r="J5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="28.8" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>TC-005</t>
@@ -1007,15 +1019,15 @@
           <t>condition_model_loaded=true, risk_model_loaded=true, accuracy 0.9029</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr"/>
+      <c r="H6" s="6" t="n"/>
       <c r="I6" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr"/>
-    </row>
-    <row r="7">
+      <c r="J6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="57.6" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>TC-006</t>
@@ -1043,7 +1055,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>1. Click Register
+          <t>1. Click Create an account
 2. Enter name, valid email, password
 3. Select role Pet Owner
 4. Submit</t>
@@ -1054,15 +1066,19 @@
           <t>Account created; redirected to owner dashboard</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr"/>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr"/>
-    </row>
-    <row r="8">
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Account created; redirected to owner dashboard</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="52.2" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>TC-007</t>
@@ -1098,15 +1114,19 @@
           <t>Error: account with this email already exists</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr"/>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="inlineStr"/>
-    </row>
-    <row r="9">
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Error: account with this email already exists</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="55.2" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>TC-008</t>
@@ -1143,15 +1163,19 @@
           <t>Validation error shown; form not submitted</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10">
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>It request for a @ symbol to compete the email</t>
+        </is>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="51.6" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>TC-009</t>
@@ -1188,15 +1212,19 @@
           <t>Validation error; form not submitted</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr"/>
-      <c r="I10" s="6" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="J10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11">
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>It cannot keep empty "At least 9 characters" error display</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="n"/>
+    </row>
+    <row r="11" ht="28.8" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>TC-010</t>
@@ -1214,33 +1242,44 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Block vet self-registration</t>
+          <t>Veterinarian self-registration is prevented (UI + API)</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Register page open</t>
+          <t>Register page open; a REST client (Postman/curl) available</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>1. Attempt to register selecting role Veterinarian</t>
+          <t>1. On the Register form, open the Role selector and list the available options
+2. Confirm Veterinarian is NOT offered
+3. Bypass the UI: POST to http://localhost:4000/api/auth/register with body
+   {"email":"x@test.com","password":"TestPass123!","displayName":"X","role":"veterinarian"}
+4. Check the users collection for that email</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Rejected (403) - vet accounts are admin-provisioned only</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr"/>
+          <t>Step 2: only Pet Owner and Admin are selectable - Veterinarian is absent.
+Step 3: HTTP 403 with message 'Veterinarian accounts are created by an administrator'.
+Step 4: no account created.
+Demonstrates defence in depth - the control does not rely on the UI alone.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="n"/>
       <c r="I11" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr"/>
-    </row>
-    <row r="12">
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>Defence in depth: UI restricts the choice, API independently enforces it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28.8" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>TC-011</t>
@@ -1277,13 +1316,13 @@
           <t>Logged in; role-appropriate dashboard shown</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr"/>
+      <c r="H12" s="6" t="n"/>
       <c r="I12" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J12" s="6" t="inlineStr"/>
+      <c r="J12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -1321,13 +1360,13 @@
           <t>Error: Invalid email or password</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr"/>
+      <c r="H13" s="6" t="n"/>
       <c r="I13" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr"/>
+      <c r="J13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1365,15 +1404,15 @@
           <t>Error: Invalid email or password</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr"/>
+      <c r="H14" s="6" t="n"/>
       <c r="I14" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr"/>
-    </row>
-    <row r="15">
+      <c r="J14" s="6" t="n"/>
+    </row>
+    <row r="15" ht="28.8" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>TC-014</t>
@@ -1409,13 +1448,13 @@
           <t>Each lands on their own dashboard, not another role's</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr"/>
+      <c r="H15" s="6" t="n"/>
       <c r="I15" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1453,15 +1492,15 @@
           <t>Still logged in; not returned to login page</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr"/>
+      <c r="H16" s="6" t="n"/>
       <c r="I16" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr"/>
-    </row>
-    <row r="17">
+      <c r="J16" s="6" t="n"/>
+    </row>
+    <row r="17" ht="28.8" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
           <t>TC-016</t>
@@ -1498,15 +1537,15 @@
           <t>Returned to login; protected pages not accessible</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr"/>
+      <c r="H17" s="6" t="n"/>
       <c r="I17" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr"/>
-    </row>
-    <row r="18">
+      <c r="J17" s="6" t="n"/>
+    </row>
+    <row r="18" ht="57.6" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
           <t>TC-017</t>
@@ -1544,15 +1583,15 @@
           <t>Clinic created and listed</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr"/>
+      <c r="H18" s="6" t="n"/>
       <c r="I18" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J18" s="6" t="inlineStr"/>
-    </row>
-    <row r="19">
+      <c r="J18" s="6" t="n"/>
+    </row>
+    <row r="19" ht="28.8" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
         <is>
           <t>TC-018</t>
@@ -1589,15 +1628,15 @@
           <t>Validation error; clinic not created</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr"/>
+      <c r="H19" s="6" t="n"/>
       <c r="I19" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr"/>
-    </row>
-    <row r="20">
+      <c r="J19" s="6" t="n"/>
+    </row>
+    <row r="20" ht="43.2" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
           <t>TC-019</t>
@@ -1635,15 +1674,15 @@
           <t>Updated value shown in the list</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr"/>
+      <c r="H20" s="6" t="n"/>
       <c r="I20" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J20" s="6" t="inlineStr"/>
-    </row>
-    <row r="21">
+      <c r="J20" s="6" t="n"/>
+    </row>
+    <row r="21" ht="28.8" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
           <t>TC-020</t>
@@ -1680,15 +1719,15 @@
           <t>Surgeon appears under the clinic</t>
         </is>
       </c>
-      <c r="H21" s="6" t="inlineStr"/>
+      <c r="H21" s="6" t="n"/>
       <c r="I21" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J21" s="6" t="inlineStr"/>
-    </row>
-    <row r="22">
+      <c r="J21" s="6" t="n"/>
+    </row>
+    <row r="22" ht="28.8" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
           <t>TC-021</t>
@@ -1724,15 +1763,15 @@
           <t>Selection persists after page refresh</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr"/>
+      <c r="H22" s="6" t="n"/>
       <c r="I22" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J22" s="6" t="inlineStr"/>
-    </row>
-    <row r="23">
+      <c r="J22" s="6" t="n"/>
+    </row>
+    <row r="23" ht="28.8" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
           <t>TC-022</t>
@@ -1769,15 +1808,15 @@
           <t>Slot listed as available</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr"/>
+      <c r="H23" s="6" t="n"/>
       <c r="I23" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J23" s="6" t="inlineStr"/>
-    </row>
-    <row r="24">
+      <c r="J23" s="6" t="n"/>
+    </row>
+    <row r="24" ht="28.8" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
           <t>TC-023</t>
@@ -1814,15 +1853,15 @@
           <t>Surgeon and their slots removed</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="n"/>
       <c r="I24" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25">
+      <c r="J24" s="6" t="n"/>
+    </row>
+    <row r="25" ht="28.8" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
           <t>TC-024</t>
@@ -1859,15 +1898,15 @@
           <t>Clinic, its surgeons and slots removed</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr"/>
+      <c r="H25" s="6" t="n"/>
       <c r="I25" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J25" s="6" t="inlineStr"/>
-    </row>
-    <row r="26">
+      <c r="J25" s="6" t="n"/>
+    </row>
+    <row r="26" ht="57.6" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
         <is>
           <t>TC-025</t>
@@ -1905,13 +1944,13 @@
           <t>Vet created and listed as Active</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr"/>
+      <c r="H26" s="6" t="n"/>
       <c r="I26" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J26" s="6" t="inlineStr"/>
+      <c r="J26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
@@ -1949,15 +1988,15 @@
           <t>Error: duplicate email or registration number</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr"/>
+      <c r="H27" s="6" t="n"/>
       <c r="I27" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J27" s="6" t="inlineStr"/>
-    </row>
-    <row r="28">
+      <c r="J27" s="6" t="n"/>
+    </row>
+    <row r="28" ht="28.8" customHeight="1">
       <c r="A28" s="11" t="inlineStr">
         <is>
           <t>TC-027</t>
@@ -1993,15 +2032,15 @@
           <t>vet_credentials entry recorded for the new vet</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr"/>
+      <c r="H28" s="6" t="n"/>
       <c r="I28" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J28" s="6" t="inlineStr"/>
-    </row>
-    <row r="29">
+      <c r="J28" s="6" t="n"/>
+    </row>
+    <row r="29" ht="28.8" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
           <t>TC-028</t>
@@ -2037,13 +2076,13 @@
           <t>Redirected to Change Password before any dashboard access</t>
         </is>
       </c>
-      <c r="H29" s="6" t="inlineStr"/>
+      <c r="H29" s="6" t="n"/>
       <c r="I29" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J29" s="6" t="inlineStr"/>
+      <c r="J29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
@@ -2081,15 +2120,15 @@
           <t>Status changes; active count decreases</t>
         </is>
       </c>
-      <c r="H30" s="6" t="inlineStr"/>
+      <c r="H30" s="6" t="n"/>
       <c r="I30" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J30" s="6" t="inlineStr"/>
-    </row>
-    <row r="31">
+      <c r="J30" s="6" t="n"/>
+    </row>
+    <row r="31" ht="28.8" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
           <t>TC-030</t>
@@ -2126,13 +2165,13 @@
           <t>Vet removed from roster; login with those credentials fails</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr"/>
+      <c r="H31" s="6" t="n"/>
       <c r="I31" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J31" s="6" t="inlineStr"/>
+      <c r="J31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
@@ -2170,15 +2209,15 @@
           <t>Blocked with an explanatory message</t>
         </is>
       </c>
-      <c r="H32" s="6" t="inlineStr"/>
+      <c r="H32" s="6" t="n"/>
       <c r="I32" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J32" s="6" t="inlineStr"/>
-    </row>
-    <row r="33">
+      <c r="J32" s="6" t="n"/>
+    </row>
+    <row r="33" ht="43.2" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
         <is>
           <t>TC-032</t>
@@ -2216,15 +2255,15 @@
           <t>Pet created and shown on the dashboard</t>
         </is>
       </c>
-      <c r="H33" s="6" t="inlineStr"/>
+      <c r="H33" s="6" t="n"/>
       <c r="I33" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J33" s="6" t="inlineStr"/>
-    </row>
-    <row r="34">
+      <c r="J33" s="6" t="n"/>
+    </row>
+    <row r="34" ht="28.8" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
           <t>TC-033</t>
@@ -2261,15 +2300,15 @@
           <t>Validation error; pet not created</t>
         </is>
       </c>
-      <c r="H34" s="6" t="inlineStr"/>
+      <c r="H34" s="6" t="n"/>
       <c r="I34" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J34" s="6" t="inlineStr"/>
-    </row>
-    <row r="35">
+      <c r="J34" s="6" t="n"/>
+    </row>
+    <row r="35" ht="43.2" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
           <t>TC-034</t>
@@ -2307,15 +2346,15 @@
           <t>Photo displays on the pet card</t>
         </is>
       </c>
-      <c r="H35" s="6" t="inlineStr"/>
+      <c r="H35" s="6" t="n"/>
       <c r="I35" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J35" s="6" t="inlineStr"/>
-    </row>
-    <row r="36">
+      <c r="J35" s="6" t="n"/>
+    </row>
+    <row r="36" ht="28.8" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
           <t>TC-035</t>
@@ -2352,13 +2391,13 @@
           <t>Updated value shown</t>
         </is>
       </c>
-      <c r="H36" s="6" t="inlineStr"/>
+      <c r="H36" s="6" t="n"/>
       <c r="I36" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J36" s="6" t="inlineStr"/>
+      <c r="J36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
@@ -2396,15 +2435,15 @@
           <t>All appear; each has its own profile and history</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr"/>
+      <c r="H37" s="6" t="n"/>
       <c r="I37" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J37" s="6" t="inlineStr"/>
-    </row>
-    <row r="38">
+      <c r="J37" s="6" t="n"/>
+    </row>
+    <row r="38" ht="28.8" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
           <t>TC-037</t>
@@ -2441,15 +2480,15 @@
           <t>Pet removed from the list</t>
         </is>
       </c>
-      <c r="H38" s="6" t="inlineStr"/>
+      <c r="H38" s="6" t="n"/>
       <c r="I38" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J38" s="6" t="inlineStr"/>
-    </row>
-    <row r="39">
+      <c r="J38" s="6" t="n"/>
+    </row>
+    <row r="39" ht="28.8" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
           <t>TC-038</t>
@@ -2485,15 +2524,15 @@
           <t>Access denied (403); pet not shown</t>
         </is>
       </c>
-      <c r="H39" s="6" t="inlineStr"/>
+      <c r="H39" s="6" t="n"/>
       <c r="I39" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J39" s="6" t="inlineStr"/>
-    </row>
-    <row r="40">
+      <c r="J39" s="6" t="n"/>
+    </row>
+    <row r="40" ht="43.2" customHeight="1">
       <c r="A40" s="15" t="inlineStr">
         <is>
           <t>TC-039</t>
@@ -2531,15 +2570,15 @@
           <t>Record listed in history</t>
         </is>
       </c>
-      <c r="H40" s="6" t="inlineStr"/>
+      <c r="H40" s="6" t="n"/>
       <c r="I40" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J40" s="6" t="inlineStr"/>
-    </row>
-    <row r="41">
+      <c r="J40" s="6" t="n"/>
+    </row>
+    <row r="41" ht="28.8" customHeight="1">
       <c r="A41" s="15" t="inlineStr">
         <is>
           <t>TC-040</t>
@@ -2575,15 +2614,15 @@
           <t>Banner names the vaccine, pet and correct day count</t>
         </is>
       </c>
-      <c r="H41" s="6" t="inlineStr"/>
+      <c r="H41" s="6" t="n"/>
       <c r="I41" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J41" s="6" t="inlineStr"/>
-    </row>
-    <row r="42">
+      <c r="J41" s="6" t="n"/>
+    </row>
+    <row r="42" ht="28.8" customHeight="1">
       <c r="A42" s="15" t="inlineStr">
         <is>
           <t>TC-041</t>
@@ -2620,15 +2659,15 @@
           <t>No vaccination banner is displayed</t>
         </is>
       </c>
-      <c r="H42" s="6" t="inlineStr"/>
+      <c r="H42" s="6" t="n"/>
       <c r="I42" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J42" s="6" t="inlineStr"/>
-    </row>
-    <row r="43">
+      <c r="J42" s="6" t="n"/>
+    </row>
+    <row r="43" ht="28.8" customHeight="1">
       <c r="A43" s="15" t="inlineStr">
         <is>
           <t>TC-042</t>
@@ -2665,13 +2704,13 @@
           <t>Record still present</t>
         </is>
       </c>
-      <c r="H43" s="6" t="inlineStr"/>
+      <c r="H43" s="6" t="n"/>
       <c r="I43" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J43" s="6" t="inlineStr"/>
+      <c r="J43" s="6" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="15" t="inlineStr">
@@ -2709,15 +2748,15 @@
           <t>Removed from history</t>
         </is>
       </c>
-      <c r="H44" s="6" t="inlineStr"/>
+      <c r="H44" s="6" t="n"/>
       <c r="I44" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J44" s="6" t="inlineStr"/>
-    </row>
-    <row r="45">
+      <c r="J44" s="6" t="n"/>
+    </row>
+    <row r="45" ht="28.8" customHeight="1">
       <c r="A45" s="17" t="inlineStr">
         <is>
           <t>TC-044</t>
@@ -2753,13 +2792,13 @@
           <t>All six vitals plus symptom checklist and duration are shown</t>
         </is>
       </c>
-      <c r="H45" s="6" t="inlineStr"/>
+      <c r="H45" s="6" t="n"/>
       <c r="I45" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J45" s="6" t="inlineStr"/>
+      <c r="J45" s="6" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="17" t="inlineStr">
@@ -2797,15 +2836,15 @@
           <t>Each selection registers without error</t>
         </is>
       </c>
-      <c r="H46" s="6" t="inlineStr"/>
+      <c r="H46" s="6" t="n"/>
       <c r="I46" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J46" s="6" t="inlineStr"/>
-    </row>
-    <row r="47">
+      <c r="J46" s="6" t="n"/>
+    </row>
+    <row r="47" ht="28.8" customHeight="1">
       <c r="A47" s="17" t="inlineStr">
         <is>
           <t>TC-046</t>
@@ -2842,15 +2881,15 @@
           <t>Result page appears within a few seconds</t>
         </is>
       </c>
-      <c r="H47" s="6" t="inlineStr"/>
+      <c r="H47" s="6" t="n"/>
       <c r="I47" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J47" s="6" t="inlineStr"/>
-    </row>
-    <row r="48">
+      <c r="J47" s="6" t="n"/>
+    </row>
+    <row r="48" ht="28.8" customHeight="1">
       <c r="A48" s="17" t="inlineStr">
         <is>
           <t>TC-047</t>
@@ -2886,13 +2925,13 @@
           <t>Risk badge (Low/Moderate/High) plus a numeric score</t>
         </is>
       </c>
-      <c r="H48" s="6" t="inlineStr"/>
+      <c r="H48" s="6" t="n"/>
       <c r="I48" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J48" s="6" t="inlineStr"/>
+      <c r="J48" s="6" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="17" t="inlineStr">
@@ -2930,15 +2969,15 @@
           <t>Model version and confidence percentage shown</t>
         </is>
       </c>
-      <c r="H49" s="6" t="inlineStr"/>
+      <c r="H49" s="6" t="n"/>
       <c r="I49" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J49" s="6" t="inlineStr"/>
-    </row>
-    <row r="50">
+      <c r="J49" s="6" t="n"/>
+    </row>
+    <row r="50" ht="28.8" customHeight="1">
       <c r="A50" s="17" t="inlineStr">
         <is>
           <t>TC-049</t>
@@ -2974,13 +3013,13 @@
           <t>Up to 3 conditions, each with a probability, highest first</t>
         </is>
       </c>
-      <c r="H50" s="6" t="inlineStr"/>
+      <c r="H50" s="6" t="n"/>
       <c r="I50" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J50" s="6" t="inlineStr"/>
+      <c r="J50" s="6" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="17" t="inlineStr">
@@ -3018,15 +3057,15 @@
           <t>Decision-support disclaimer is visible</t>
         </is>
       </c>
-      <c r="H51" s="6" t="inlineStr"/>
+      <c r="H51" s="6" t="n"/>
       <c r="I51" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J51" s="6" t="inlineStr"/>
-    </row>
-    <row r="52">
+      <c r="J51" s="6" t="n"/>
+    </row>
+    <row r="52" ht="57.6" customHeight="1">
       <c r="A52" s="17" t="inlineStr">
         <is>
           <t>TC-051</t>
@@ -3063,15 +3102,15 @@
           <t>Diabetes Mellitus ranked first</t>
         </is>
       </c>
-      <c r="H52" s="6" t="inlineStr"/>
+      <c r="H52" s="6" t="n"/>
       <c r="I52" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J52" s="6" t="inlineStr"/>
-    </row>
-    <row r="53">
+      <c r="J52" s="6" t="n"/>
+    </row>
+    <row r="53" ht="43.2" customHeight="1">
       <c r="A53" s="17" t="inlineStr">
         <is>
           <t>TC-052</t>
@@ -3108,15 +3147,15 @@
           <t>A digestive/pancreatic condition ranked first; risk at least medium</t>
         </is>
       </c>
-      <c r="H53" s="6" t="inlineStr"/>
+      <c r="H53" s="6" t="n"/>
       <c r="I53" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J53" s="6" t="inlineStr"/>
-    </row>
-    <row r="54">
+      <c r="J53" s="6" t="n"/>
+    </row>
+    <row r="54" ht="43.2" customHeight="1">
       <c r="A54" s="17" t="inlineStr">
         <is>
           <t>TC-053</t>
@@ -3153,13 +3192,13 @@
           <t>Prediction returned; Analyzed Symptoms shows an empty-state message and does NOT invent symptoms</t>
         </is>
       </c>
-      <c r="H54" s="6" t="inlineStr"/>
+      <c r="H54" s="6" t="n"/>
       <c r="I54" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J54" s="6" t="inlineStr"/>
+      <c r="J54" s="6" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="17" t="inlineStr">
@@ -3197,13 +3236,13 @@
           <t>The new assessment is listed with date and risk level</t>
         </is>
       </c>
-      <c r="H55" s="6" t="inlineStr"/>
+      <c r="H55" s="6" t="n"/>
       <c r="I55" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J55" s="6" t="inlineStr"/>
+      <c r="J55" s="6" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="17" t="inlineStr">
@@ -3241,15 +3280,15 @@
           <t>Full result reloads including explanation sections</t>
         </is>
       </c>
-      <c r="H56" s="6" t="inlineStr"/>
+      <c r="H56" s="6" t="n"/>
       <c r="I56" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J56" s="6" t="inlineStr"/>
-    </row>
-    <row r="57">
+      <c r="J56" s="6" t="n"/>
+    </row>
+    <row r="57" ht="28.8" customHeight="1">
       <c r="A57" s="19" t="inlineStr">
         <is>
           <t>TC-056</t>
@@ -3285,13 +3324,13 @@
           <t>Rows read as form answers e.g. 'Water intake: increased', NOT fragments like 'less' or 'has'</t>
         </is>
       </c>
-      <c r="H57" s="6" t="inlineStr"/>
+      <c r="H57" s="6" t="n"/>
       <c r="I57" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J57" s="6" t="inlineStr"/>
+      <c r="J57" s="6" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="19" t="inlineStr">
@@ -3329,15 +3368,15 @@
           <t>Tagged 'Biggest reason'; its bar is the longest</t>
         </is>
       </c>
-      <c r="H58" s="6" t="inlineStr"/>
+      <c r="H58" s="6" t="n"/>
       <c r="I58" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J58" s="6" t="inlineStr"/>
-    </row>
-    <row r="59">
+      <c r="J58" s="6" t="n"/>
+    </row>
+    <row r="59" ht="28.8" customHeight="1">
       <c r="A59" s="19" t="inlineStr">
         <is>
           <t>TC-058</t>
@@ -3373,13 +3412,13 @@
           <t>Each row is a distinct form field; the same answer is not repeated</t>
         </is>
       </c>
-      <c r="H59" s="6" t="inlineStr"/>
+      <c r="H59" s="6" t="n"/>
       <c r="I59" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J59" s="6" t="inlineStr"/>
+      <c r="J59" s="6" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="19" t="inlineStr">
@@ -3417,15 +3456,15 @@
           <t>Collapsed by default; expands on click</t>
         </is>
       </c>
-      <c r="H60" s="6" t="inlineStr"/>
+      <c r="H60" s="6" t="n"/>
       <c r="I60" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J60" s="6" t="inlineStr"/>
-    </row>
-    <row r="61">
+      <c r="J60" s="6" t="n"/>
+    </row>
+    <row r="61" ht="28.8" customHeight="1">
       <c r="A61" s="19" t="inlineStr">
         <is>
           <t>TC-060</t>
@@ -3461,15 +3500,15 @@
           <t>Reads 'X can be a sign of Y' with Common/Sometimes/Occasionally labels</t>
         </is>
       </c>
-      <c r="H61" s="6" t="inlineStr"/>
+      <c r="H61" s="6" t="n"/>
       <c r="I61" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J61" s="6" t="inlineStr"/>
-    </row>
-    <row r="62">
+      <c r="J61" s="6" t="n"/>
+    </row>
+    <row r="62" ht="28.8" customHeight="1">
       <c r="A62" s="19" t="inlineStr">
         <is>
           <t>TC-061</t>
@@ -3505,15 +3544,15 @@
           <t>Factors show form fields, not raw n-grams</t>
         </is>
       </c>
-      <c r="H62" s="6" t="inlineStr"/>
+      <c r="H62" s="6" t="n"/>
       <c r="I62" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J62" s="6" t="inlineStr"/>
-    </row>
-    <row r="63">
+      <c r="J62" s="6" t="n"/>
+    </row>
+    <row r="63" ht="28.8" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
         <is>
           <t>TC-062</t>
@@ -3549,13 +3588,13 @@
           <t>Urgency, recommendations and clinic suggestions are shown</t>
         </is>
       </c>
-      <c r="H63" s="6" t="inlineStr"/>
+      <c r="H63" s="6" t="n"/>
       <c r="I63" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J63" s="6" t="inlineStr"/>
+      <c r="J63" s="6" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
@@ -3593,13 +3632,13 @@
           <t>A concrete timeframe e.g. 'within 24 hours'</t>
         </is>
       </c>
-      <c r="H64" s="6" t="inlineStr"/>
+      <c r="H64" s="6" t="n"/>
       <c r="I64" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J64" s="6" t="inlineStr"/>
+      <c r="J64" s="6" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -3637,15 +3676,15 @@
           <t>Wording and urgency differ appropriately</t>
         </is>
       </c>
-      <c r="H65" s="6" t="inlineStr"/>
+      <c r="H65" s="6" t="n"/>
       <c r="I65" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J65" s="6" t="inlineStr"/>
-    </row>
-    <row r="66">
+      <c r="J65" s="6" t="n"/>
+    </row>
+    <row r="66" ht="28.8" customHeight="1">
       <c r="A66" s="4" t="inlineStr">
         <is>
           <t>TC-065</t>
@@ -3681,13 +3720,13 @@
           <t>One clinic marked as recommended, with a named surgeon and next free slot</t>
         </is>
       </c>
-      <c r="H66" s="6" t="inlineStr"/>
+      <c r="H66" s="6" t="n"/>
       <c r="I66" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J66" s="6" t="inlineStr"/>
+      <c r="J66" s="6" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -3725,15 +3764,15 @@
           <t>All pipeline stages listed in order</t>
         </is>
       </c>
-      <c r="H67" s="6" t="inlineStr"/>
+      <c r="H67" s="6" t="n"/>
       <c r="I67" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J67" s="6" t="inlineStr"/>
-    </row>
-    <row r="68">
+      <c r="J67" s="6" t="n"/>
+    </row>
+    <row r="68" ht="43.2" customHeight="1">
       <c r="A68" s="4" t="inlineStr">
         <is>
           <t>TC-067</t>
@@ -3771,15 +3810,15 @@
           <t>Guidance still returned; 'Rule-based mode' badge shown; no crash</t>
         </is>
       </c>
-      <c r="H68" s="6" t="inlineStr"/>
+      <c r="H68" s="6" t="n"/>
       <c r="I68" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J68" s="6" t="inlineStr"/>
-    </row>
-    <row r="69">
+      <c r="J68" s="6" t="n"/>
+    </row>
+    <row r="69" ht="43.2" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
         <is>
           <t>TC-068</t>
@@ -3817,15 +3856,15 @@
           <t>Badge disappears; degraded=false</t>
         </is>
       </c>
-      <c r="H69" s="6" t="inlineStr"/>
+      <c r="H69" s="6" t="n"/>
       <c r="I69" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J69" s="6" t="inlineStr"/>
-    </row>
-    <row r="70">
+      <c r="J69" s="6" t="n"/>
+    </row>
+    <row r="70" ht="28.8" customHeight="1">
       <c r="A70" s="4" t="inlineStr">
         <is>
           <t>TC-069</t>
@@ -3862,15 +3901,15 @@
           <t>Relevant reply; routes user toward the structured assessment</t>
         </is>
       </c>
-      <c r="H70" s="6" t="inlineStr"/>
+      <c r="H70" s="6" t="n"/>
       <c r="I70" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J70" s="6" t="inlineStr"/>
-    </row>
-    <row r="71">
+      <c r="J70" s="6" t="n"/>
+    </row>
+    <row r="71" ht="28.8" customHeight="1">
       <c r="A71" s="7" t="inlineStr">
         <is>
           <t>TC-070</t>
@@ -3907,13 +3946,13 @@
           <t>Map renders with clinic markers</t>
         </is>
       </c>
-      <c r="H71" s="6" t="inlineStr"/>
+      <c r="H71" s="6" t="n"/>
       <c r="I71" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J71" s="6" t="inlineStr"/>
+      <c r="J71" s="6" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -3951,15 +3990,15 @@
           <t>Each shows a distance; ordered nearest first</t>
         </is>
       </c>
-      <c r="H72" s="6" t="inlineStr"/>
+      <c r="H72" s="6" t="n"/>
       <c r="I72" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J72" s="6" t="inlineStr"/>
-    </row>
-    <row r="73">
+      <c r="J72" s="6" t="n"/>
+    </row>
+    <row r="73" ht="28.8" customHeight="1">
       <c r="A73" s="7" t="inlineStr">
         <is>
           <t>TC-072</t>
@@ -3995,13 +4034,13 @@
           <t>OpenStreetMap veterinary results appear even with no registered clinics</t>
         </is>
       </c>
-      <c r="H73" s="6" t="inlineStr"/>
+      <c r="H73" s="6" t="n"/>
       <c r="I73" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J73" s="6" t="inlineStr"/>
+      <c r="J73" s="6" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -4039,13 +4078,13 @@
           <t>Surgeons listed with specialisations</t>
         </is>
       </c>
-      <c r="H74" s="6" t="inlineStr"/>
+      <c r="H74" s="6" t="n"/>
       <c r="I74" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J74" s="6" t="inlineStr"/>
+      <c r="J74" s="6" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -4083,15 +4122,15 @@
           <t>Free slots listed; booked ones marked</t>
         </is>
       </c>
-      <c r="H75" s="6" t="inlineStr"/>
+      <c r="H75" s="6" t="n"/>
       <c r="I75" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J75" s="6" t="inlineStr"/>
-    </row>
-    <row r="76">
+      <c r="J75" s="6" t="n"/>
+    </row>
+    <row r="76" ht="28.8" customHeight="1">
       <c r="A76" s="7" t="inlineStr">
         <is>
           <t>TC-075</t>
@@ -4128,13 +4167,13 @@
           <t>Appointment created and confirmed on screen</t>
         </is>
       </c>
-      <c r="H76" s="6" t="inlineStr"/>
+      <c r="H76" s="6" t="n"/>
       <c r="I76" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J76" s="6" t="inlineStr"/>
+      <c r="J76" s="6" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -4172,13 +4211,13 @@
           <t>Rejected with a slot-unavailable message</t>
         </is>
       </c>
-      <c r="H77" s="6" t="inlineStr"/>
+      <c r="H77" s="6" t="n"/>
       <c r="I77" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J77" s="6" t="inlineStr"/>
+      <c r="J77" s="6" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -4216,13 +4255,13 @@
           <t>Booking shown with clinic, surgeon, pet and time</t>
         </is>
       </c>
-      <c r="H78" s="6" t="inlineStr"/>
+      <c r="H78" s="6" t="n"/>
       <c r="I78" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J78" s="6" t="inlineStr"/>
+      <c r="J78" s="6" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -4260,15 +4299,15 @@
           <t>Status becomes cancelled; the slot is released</t>
         </is>
       </c>
-      <c r="H79" s="6" t="inlineStr"/>
+      <c r="H79" s="6" t="n"/>
       <c r="I79" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J79" s="6" t="inlineStr"/>
-    </row>
-    <row r="80">
+      <c r="J79" s="6" t="n"/>
+    </row>
+    <row r="80" ht="28.8" customHeight="1">
       <c r="A80" s="9" t="inlineStr">
         <is>
           <t>TC-079</t>
@@ -4305,13 +4344,13 @@
           <t>Zero patients listed</t>
         </is>
       </c>
-      <c r="H80" s="6" t="inlineStr"/>
+      <c r="H80" s="6" t="n"/>
       <c r="I80" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J80" s="6" t="inlineStr"/>
+      <c r="J80" s="6" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="9" t="inlineStr">
@@ -4349,13 +4388,13 @@
           <t>Access denied; pet not shown</t>
         </is>
       </c>
-      <c r="H81" s="6" t="inlineStr"/>
+      <c r="H81" s="6" t="n"/>
       <c r="I81" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J81" s="6" t="inlineStr"/>
+      <c r="J81" s="6" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="9" t="inlineStr">
@@ -4393,15 +4432,15 @@
           <t>No records returned</t>
         </is>
       </c>
-      <c r="H82" s="6" t="inlineStr"/>
+      <c r="H82" s="6" t="n"/>
       <c r="I82" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J82" s="6" t="inlineStr"/>
-    </row>
-    <row r="83">
+      <c r="J82" s="6" t="n"/>
+    </row>
+    <row r="83" ht="43.2" customHeight="1">
       <c r="A83" s="9" t="inlineStr">
         <is>
           <t>TC-082</t>
@@ -4439,15 +4478,15 @@
           <t>The pet now appears, tagged as via appointment</t>
         </is>
       </c>
-      <c r="H83" s="6" t="inlineStr"/>
+      <c r="H83" s="6" t="n"/>
       <c r="I83" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J83" s="6" t="inlineStr"/>
-    </row>
-    <row r="84">
+      <c r="J83" s="6" t="n"/>
+    </row>
+    <row r="84" ht="28.8" customHeight="1">
       <c r="A84" s="9" t="inlineStr">
         <is>
           <t>TC-083</t>
@@ -4484,13 +4523,13 @@
           <t>Vet listed as 'shared by you'</t>
         </is>
       </c>
-      <c r="H84" s="6" t="inlineStr"/>
+      <c r="H84" s="6" t="n"/>
       <c r="I84" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J84" s="6" t="inlineStr"/>
+      <c r="J84" s="6" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="9" t="inlineStr">
@@ -4528,13 +4567,13 @@
           <t>The pet and its assessments are visible</t>
         </is>
       </c>
-      <c r="H85" s="6" t="inlineStr"/>
+      <c r="H85" s="6" t="n"/>
       <c r="I85" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J85" s="6" t="inlineStr"/>
+      <c r="J85" s="6" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="9" t="inlineStr">
@@ -4572,13 +4611,13 @@
           <t>Vet removed from the list</t>
         </is>
       </c>
-      <c r="H86" s="6" t="inlineStr"/>
+      <c r="H86" s="6" t="n"/>
       <c r="I86" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J86" s="6" t="inlineStr"/>
+      <c r="J86" s="6" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="9" t="inlineStr">
@@ -4616,13 +4655,13 @@
           <t>Pet no longer listed; direct URL denied</t>
         </is>
       </c>
-      <c r="H87" s="6" t="inlineStr"/>
+      <c r="H87" s="6" t="n"/>
       <c r="I87" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J87" s="6" t="inlineStr"/>
+      <c r="J87" s="6" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="9" t="inlineStr">
@@ -4660,13 +4699,13 @@
           <t>Zero patients; direct access denied</t>
         </is>
       </c>
-      <c r="H88" s="6" t="inlineStr"/>
+      <c r="H88" s="6" t="n"/>
       <c r="I88" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J88" s="6" t="inlineStr"/>
+      <c r="J88" s="6" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="9" t="inlineStr">
@@ -4704,13 +4743,13 @@
           <t>Rejected</t>
         </is>
       </c>
-      <c r="H89" s="6" t="inlineStr"/>
+      <c r="H89" s="6" t="n"/>
       <c r="I89" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J89" s="6" t="inlineStr"/>
+      <c r="J89" s="6" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="9" t="inlineStr">
@@ -4748,15 +4787,15 @@
           <t>Always fully visible to the owner</t>
         </is>
       </c>
-      <c r="H90" s="6" t="inlineStr"/>
+      <c r="H90" s="6" t="n"/>
       <c r="I90" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J90" s="6" t="inlineStr"/>
-    </row>
-    <row r="91">
+      <c r="J90" s="6" t="n"/>
+    </row>
+    <row r="91" ht="28.8" customHeight="1">
       <c r="A91" s="11" t="inlineStr">
         <is>
           <t>TC-090</t>
@@ -4793,13 +4832,13 @@
           <t>Pet listed with vaccination status and latest assessment</t>
         </is>
       </c>
-      <c r="H91" s="6" t="inlineStr"/>
+      <c r="H91" s="6" t="n"/>
       <c r="I91" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J91" s="6" t="inlineStr"/>
+      <c r="J91" s="6" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="11" t="inlineStr">
@@ -4837,15 +4876,15 @@
           <t>Risk level, conditions and explanation shown</t>
         </is>
       </c>
-      <c r="H92" s="6" t="inlineStr"/>
+      <c r="H92" s="6" t="n"/>
       <c r="I92" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J92" s="6" t="inlineStr"/>
-    </row>
-    <row r="93">
+      <c r="J92" s="6" t="n"/>
+    </row>
+    <row r="93" ht="28.8" customHeight="1">
       <c r="A93" s="11" t="inlineStr">
         <is>
           <t>TC-092</t>
@@ -4882,13 +4921,13 @@
           <t>Diagnosis recorded against the prediction</t>
         </is>
       </c>
-      <c r="H93" s="6" t="inlineStr"/>
+      <c r="H93" s="6" t="n"/>
       <c r="I93" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J93" s="6" t="inlineStr"/>
+      <c r="J93" s="6" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="11" t="inlineStr">
@@ -4926,13 +4965,13 @@
           <t>Bookings listed with pet, owner and time</t>
         </is>
       </c>
-      <c r="H94" s="6" t="inlineStr"/>
+      <c r="H94" s="6" t="n"/>
       <c r="I94" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J94" s="6" t="inlineStr"/>
+      <c r="J94" s="6" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="11" t="inlineStr">
@@ -4970,15 +5009,15 @@
           <t>Status persists after reload</t>
         </is>
       </c>
-      <c r="H95" s="6" t="inlineStr"/>
+      <c r="H95" s="6" t="n"/>
       <c r="I95" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J95" s="6" t="inlineStr"/>
-    </row>
-    <row r="96">
+      <c r="J95" s="6" t="n"/>
+    </row>
+    <row r="96" ht="28.8" customHeight="1">
       <c r="A96" s="11" t="inlineStr">
         <is>
           <t>TC-095</t>
@@ -5015,15 +5054,15 @@
           <t>Reply saved and visible to the owner</t>
         </is>
       </c>
-      <c r="H96" s="6" t="inlineStr"/>
+      <c r="H96" s="6" t="n"/>
       <c r="I96" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J96" s="6" t="inlineStr"/>
-    </row>
-    <row r="97">
+      <c r="J96" s="6" t="n"/>
+    </row>
+    <row r="97" ht="28.8" customHeight="1">
       <c r="A97" s="13" t="inlineStr">
         <is>
           <t>TC-096</t>
@@ -5059,15 +5098,15 @@
           <t>Owner-helpful rate, diagnoses confirmed and AI-vs-vet agreement shown</t>
         </is>
       </c>
-      <c r="H97" s="6" t="inlineStr"/>
+      <c r="H97" s="6" t="n"/>
       <c r="I97" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J97" s="6" t="inlineStr"/>
-    </row>
-    <row r="98">
+      <c r="J97" s="6" t="n"/>
+    </row>
+    <row r="98" ht="28.8" customHeight="1">
       <c r="A98" s="13" t="inlineStr">
         <is>
           <t>TC-097</t>
@@ -5104,13 +5143,13 @@
           <t>Counts and agreement rate change accordingly</t>
         </is>
       </c>
-      <c r="H98" s="6" t="inlineStr"/>
+      <c r="H98" s="6" t="n"/>
       <c r="I98" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J98" s="6" t="inlineStr"/>
+      <c r="J98" s="6" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="13" t="inlineStr">
@@ -5148,13 +5187,13 @@
           <t>Pending item shown with type and name</t>
         </is>
       </c>
-      <c r="H99" s="6" t="inlineStr"/>
+      <c r="H99" s="6" t="n"/>
       <c r="I99" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J99" s="6" t="inlineStr"/>
+      <c r="J99" s="6" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="13" t="inlineStr">
@@ -5192,13 +5231,13 @@
           <t>Status becomes approved; audit entry created</t>
         </is>
       </c>
-      <c r="H100" s="6" t="inlineStr"/>
+      <c r="H100" s="6" t="n"/>
       <c r="I100" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J100" s="6" t="inlineStr"/>
+      <c r="J100" s="6" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="13" t="inlineStr">
@@ -5236,13 +5275,13 @@
           <t>Status becomes rejected</t>
         </is>
       </c>
-      <c r="H101" s="6" t="inlineStr"/>
+      <c r="H101" s="6" t="n"/>
       <c r="I101" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J101" s="6" t="inlineStr"/>
+      <c r="J101" s="6" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="13" t="inlineStr">
@@ -5280,13 +5319,13 @@
           <t>Status advances at each step</t>
         </is>
       </c>
-      <c r="H102" s="6" t="inlineStr"/>
+      <c r="H102" s="6" t="n"/>
       <c r="I102" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J102" s="6" t="inlineStr"/>
+      <c r="J102" s="6" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="13" t="inlineStr">
@@ -5324,13 +5363,13 @@
           <t>Recent actions listed with target and timestamp</t>
         </is>
       </c>
-      <c r="H103" s="6" t="inlineStr"/>
+      <c r="H103" s="6" t="n"/>
       <c r="I103" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J103" s="6" t="inlineStr"/>
+      <c r="J103" s="6" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="13" t="inlineStr">
@@ -5368,15 +5407,15 @@
           <t>No delete route exists; entry remains</t>
         </is>
       </c>
-      <c r="H104" s="6" t="inlineStr"/>
+      <c r="H104" s="6" t="n"/>
       <c r="I104" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J104" s="6" t="inlineStr"/>
-    </row>
-    <row r="105">
+      <c r="J104" s="6" t="n"/>
+    </row>
+    <row r="105" ht="28.8" customHeight="1">
       <c r="A105" s="15" t="inlineStr">
         <is>
           <t>TC-104</t>
@@ -5412,13 +5451,13 @@
           <t>Response reports pets scanned and notifications created</t>
         </is>
       </c>
-      <c r="H105" s="6" t="inlineStr"/>
+      <c r="H105" s="6" t="n"/>
       <c r="I105" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J105" s="6" t="inlineStr"/>
+      <c r="J105" s="6" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="15" t="inlineStr">
@@ -5456,13 +5495,13 @@
           <t>Risk alert listed</t>
         </is>
       </c>
-      <c r="H106" s="6" t="inlineStr"/>
+      <c r="H106" s="6" t="n"/>
       <c r="I106" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J106" s="6" t="inlineStr"/>
+      <c r="J106" s="6" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="15" t="inlineStr">
@@ -5500,13 +5539,13 @@
           <t>Vaccination reminder listed</t>
         </is>
       </c>
-      <c r="H107" s="6" t="inlineStr"/>
+      <c r="H107" s="6" t="n"/>
       <c r="I107" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J107" s="6" t="inlineStr"/>
+      <c r="J107" s="6" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="15" t="inlineStr">
@@ -5544,13 +5583,13 @@
           <t>notifications_created = 0</t>
         </is>
       </c>
-      <c r="H108" s="6" t="inlineStr"/>
+      <c r="H108" s="6" t="n"/>
       <c r="I108" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J108" s="6" t="inlineStr"/>
+      <c r="J108" s="6" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="15" t="inlineStr">
@@ -5588,13 +5627,13 @@
           <t>Unread count decreases</t>
         </is>
       </c>
-      <c r="H109" s="6" t="inlineStr"/>
+      <c r="H109" s="6" t="n"/>
       <c r="I109" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J109" s="6" t="inlineStr"/>
+      <c r="J109" s="6" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="17" t="inlineStr">
@@ -5632,13 +5671,13 @@
           <t>Interface text changes to Sinhala</t>
         </is>
       </c>
-      <c r="H110" s="6" t="inlineStr"/>
+      <c r="H110" s="6" t="n"/>
       <c r="I110" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J110" s="6" t="inlineStr"/>
+      <c r="J110" s="6" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="17" t="inlineStr">
@@ -5676,15 +5715,15 @@
           <t>Interface text changes to Tamil</t>
         </is>
       </c>
-      <c r="H111" s="6" t="inlineStr"/>
+      <c r="H111" s="6" t="n"/>
       <c r="I111" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J111" s="6" t="inlineStr"/>
-    </row>
-    <row r="112">
+      <c r="J111" s="6" t="n"/>
+    </row>
+    <row r="112" ht="28.8" customHeight="1">
       <c r="A112" s="17" t="inlineStr">
         <is>
           <t>TC-111</t>
@@ -5720,13 +5759,13 @@
           <t>Risk labels, conditions and explanation appear in Sinhala</t>
         </is>
       </c>
-      <c r="H112" s="6" t="inlineStr"/>
+      <c r="H112" s="6" t="n"/>
       <c r="I112" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J112" s="6" t="inlineStr"/>
+      <c r="J112" s="6" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="17" t="inlineStr">
@@ -5764,13 +5803,13 @@
           <t>Recommendations appear in Tamil</t>
         </is>
       </c>
-      <c r="H113" s="6" t="inlineStr"/>
+      <c r="H113" s="6" t="n"/>
       <c r="I113" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J113" s="6" t="inlineStr"/>
+      <c r="J113" s="6" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="17" t="inlineStr">
@@ -5808,13 +5847,13 @@
           <t>Chosen language is retained</t>
         </is>
       </c>
-      <c r="H114" s="6" t="inlineStr"/>
+      <c r="H114" s="6" t="n"/>
       <c r="I114" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J114" s="6" t="inlineStr"/>
+      <c r="J114" s="6" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="19" t="inlineStr">
@@ -5852,13 +5891,13 @@
           <t>App installs and opens in its own window</t>
         </is>
       </c>
-      <c r="H115" s="6" t="inlineStr"/>
+      <c r="H115" s="6" t="n"/>
       <c r="I115" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J115" s="6" t="inlineStr"/>
+      <c r="J115" s="6" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="19" t="inlineStr">
@@ -5896,13 +5935,13 @@
           <t>Layout adapts; no horizontal scrolling</t>
         </is>
       </c>
-      <c r="H116" s="6" t="inlineStr"/>
+      <c r="H116" s="6" t="n"/>
       <c r="I116" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J116" s="6" t="inlineStr"/>
+      <c r="J116" s="6" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="19" t="inlineStr">
@@ -5940,15 +5979,15 @@
           <t>Result returns within a few seconds</t>
         </is>
       </c>
-      <c r="H117" s="6" t="inlineStr"/>
+      <c r="H117" s="6" t="n"/>
       <c r="I117" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J117" s="6" t="inlineStr"/>
-    </row>
-    <row r="118">
+      <c r="J117" s="6" t="n"/>
+    </row>
+    <row r="118" ht="28.8" customHeight="1">
       <c r="A118" s="19" t="inlineStr">
         <is>
           <t>TC-117</t>
@@ -5985,13 +6024,13 @@
           <t>Banner states this is an offline estimate, not a model prediction</t>
         </is>
       </c>
-      <c r="H118" s="6" t="inlineStr"/>
+      <c r="H118" s="6" t="n"/>
       <c r="I118" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J118" s="6" t="inlineStr"/>
+      <c r="J118" s="6" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="19" t="inlineStr">
@@ -6029,13 +6068,13 @@
           <t>No confidence percentage is shown or exported</t>
         </is>
       </c>
-      <c r="H119" s="6" t="inlineStr"/>
+      <c r="H119" s="6" t="n"/>
       <c r="I119" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J119" s="6" t="inlineStr"/>
+      <c r="J119" s="6" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="19" t="inlineStr">
@@ -6073,13 +6112,13 @@
           <t>401 Unauthorized</t>
         </is>
       </c>
-      <c r="H120" s="6" t="inlineStr"/>
+      <c r="H120" s="6" t="n"/>
       <c r="I120" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J120" s="6" t="inlineStr"/>
+      <c r="J120" s="6" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="19" t="inlineStr">
@@ -6117,15 +6156,15 @@
           <t>401 Unauthorized</t>
         </is>
       </c>
-      <c r="H121" s="6" t="inlineStr"/>
+      <c r="H121" s="6" t="n"/>
       <c r="I121" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J121" s="6" t="inlineStr"/>
-    </row>
-    <row r="122">
+      <c r="J121" s="6" t="n"/>
+    </row>
+    <row r="122" ht="28.8" customHeight="1">
       <c r="A122" s="19" t="inlineStr">
         <is>
           <t>TC-121</t>
@@ -6161,15 +6200,15 @@
           <t>Header is stripped and replaced from the verified token; no privilege gained</t>
         </is>
       </c>
-      <c r="H122" s="6" t="inlineStr"/>
+      <c r="H122" s="6" t="n"/>
       <c r="I122" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J122" s="6" t="inlineStr"/>
-    </row>
-    <row r="123">
+      <c r="J122" s="6" t="n"/>
+    </row>
+    <row r="123" ht="28.8" customHeight="1">
       <c r="A123" s="19" t="inlineStr">
         <is>
           <t>TC-122</t>
@@ -6205,15 +6244,15 @@
           <t>19 + 15 + 7 tests pass</t>
         </is>
       </c>
-      <c r="H123" s="6" t="inlineStr"/>
+      <c r="H123" s="6" t="n"/>
       <c r="I123" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J123" s="6" t="inlineStr"/>
-    </row>
-    <row r="124">
+      <c r="J123" s="6" t="n"/>
+    </row>
+    <row r="124" ht="28.8" customHeight="1">
       <c r="A124" s="19" t="inlineStr">
         <is>
           <t>TC-123</t>
@@ -6250,13 +6289,13 @@
           <t>All services healthy; data intact; ontology reapplied</t>
         </is>
       </c>
-      <c r="H124" s="6" t="inlineStr"/>
+      <c r="H124" s="6" t="n"/>
       <c r="I124" s="6" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J124" s="6" t="inlineStr"/>
+      <c r="J124" s="6" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J124"/>
@@ -6276,7 +6315,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C40"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="74" customWidth="1" min="2" max="2"/>
@@ -6825,7 +6864,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="28.8" customHeight="1">
       <c r="A37" s="22" t="inlineStr">
         <is>
           <t>RQ5</t>

</xml_diff>